<commit_message>
all features now work with the format+ improving left and right margin with segmentation
</commit_message>
<xml_diff>
--- a/FinalFeatureExtraction/tables/bottom_margin.xlsx
+++ b/FinalFeatureExtraction/tables/bottom_margin.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,11 +443,161 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sd_COLUMNS.png</t>
+          <t>SaraRosenboum_COLUMNS.png</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4769</v>
+        <v>0.3034</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan1_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.7702</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>izhak_rosenboum_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.9444</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>scan 10_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>scan 9_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>scan11_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>scan12_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.5402</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>scan13_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1046</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>scan14_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.6153</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>scan2_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.9425</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>scan3_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3947</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>scan4_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1731</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>scan5_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>scan6_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.582</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>scan7_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2758</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>scan8_COLUMNS.png</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.9596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed some feature to calculate mean instead of median. and updated prompt
</commit_message>
<xml_diff>
--- a/FinalFeatureExtraction/tables/bottom_margin.xlsx
+++ b/FinalFeatureExtraction/tables/bottom_margin.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,161 +443,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SaraRosenboum_COLUMNS.png</t>
+          <t>izhak_rosenboum_COLUMNS.png</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3034</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Scan1_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.7702</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>izhak_rosenboum_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
         <v>0.9444</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>scan 10_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>scan 9_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>scan11_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>scan12_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.5402</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>scan13_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.1046</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>scan14_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.6153</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>scan2_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.9425</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>scan3_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.3947</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>scan4_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.1731</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>scan5_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>scan6_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.582</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>scan7_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.2758</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>scan8_COLUMNS.png</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.9596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>